<commit_message>
init: first import grt system
</commit_message>
<xml_diff>
--- a/data/副本GRT人员能力测评（202602）.xlsx
+++ b/data/副本GRT人员能力测评（202602）.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\history\20260210\grt-implementation-plan\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{05A7EA2C-5C4C-4117-86BB-D1FF58E3C334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B008C90-2EC5-49D3-8C91-008D55638BB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -348,9 +348,6 @@
     <t>刘坤</t>
   </si>
   <si>
-    <t>市场主管</t>
-  </si>
-  <si>
     <t>GRT087</t>
   </si>
   <si>
@@ -445,6 +442,10 @@
   </si>
   <si>
     <t>AI数智&amp;人事行政部经理</t>
+  </si>
+  <si>
+    <t>销售工程师/市场主管</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -2269,7 +2270,7 @@
         <v>91</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="E28" s="10" t="s">
         <v>15</v>
@@ -2299,13 +2300,13 @@
         <v>27</v>
       </c>
       <c r="B29" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="D29" s="10" t="s">
         <v>94</v>
-      </c>
-      <c r="D29" s="10" t="s">
-        <v>95</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>17</v>
@@ -2335,13 +2336,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="C30" s="10" t="s">
-        <v>97</v>
-      </c>
       <c r="D30" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E30" s="10" t="s">
         <v>17</v>
@@ -2371,13 +2372,13 @@
         <v>29</v>
       </c>
       <c r="B31" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C31" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="D31" s="10" t="s">
         <v>99</v>
-      </c>
-      <c r="D31" s="10" t="s">
-        <v>100</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>17</v>
@@ -2407,13 +2408,13 @@
         <v>30</v>
       </c>
       <c r="B32" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="C32" s="10" t="s">
-        <v>102</v>
-      </c>
       <c r="D32" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E32" s="10" t="s">
         <v>17</v>
@@ -2443,10 +2444,10 @@
         <v>31</v>
       </c>
       <c r="B33" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C33" s="10" t="s">
         <v>103</v>
-      </c>
-      <c r="C33" s="10" t="s">
-        <v>104</v>
       </c>
       <c r="D33" s="10" t="s">
         <v>38</v>
@@ -2479,13 +2480,13 @@
         <v>32</v>
       </c>
       <c r="B34" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C34" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="D34" s="10" t="s">
         <v>106</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>107</v>
       </c>
       <c r="E34" s="10" t="s">
         <v>21</v>
@@ -2515,10 +2516,10 @@
         <v>33</v>
       </c>
       <c r="B35" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C35" s="10" t="s">
         <v>108</v>
-      </c>
-      <c r="C35" s="10" t="s">
-        <v>109</v>
       </c>
       <c r="D35" s="10" t="s">
         <v>34</v>
@@ -2551,10 +2552,10 @@
         <v>34</v>
       </c>
       <c r="B36" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C36" s="9" t="s">
         <v>110</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="D36" s="9" t="s">
         <v>54</v>
@@ -2587,13 +2588,13 @@
         <v>35</v>
       </c>
       <c r="B37" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C37" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="D37" s="10" t="s">
         <v>113</v>
-      </c>
-      <c r="D37" s="10" t="s">
-        <v>114</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>17</v>
@@ -2623,13 +2624,13 @@
         <v>36</v>
       </c>
       <c r="B38" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C38" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="C38" s="10" t="s">
+      <c r="D38" s="10" t="s">
         <v>116</v>
-      </c>
-      <c r="D38" s="10" t="s">
-        <v>117</v>
       </c>
       <c r="E38" s="10" t="s">
         <v>17</v>
@@ -2659,13 +2660,13 @@
         <v>37</v>
       </c>
       <c r="B39" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C39" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="D39" s="10" t="s">
         <v>119</v>
-      </c>
-      <c r="D39" s="10" t="s">
-        <v>120</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>17</v>
@@ -2695,10 +2696,10 @@
         <v>38</v>
       </c>
       <c r="B40" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C40" s="10" t="s">
         <v>121</v>
-      </c>
-      <c r="C40" s="10" t="s">
-        <v>122</v>
       </c>
       <c r="D40" s="10" t="s">
         <v>38</v>
@@ -2729,10 +2730,10 @@
       <c r="A41" s="7"/>
       <c r="B41" s="8"/>
       <c r="C41" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="D41" s="10" t="s">
         <v>123</v>
-      </c>
-      <c r="D41" s="10" t="s">
-        <v>124</v>
       </c>
       <c r="E41" s="10"/>
       <c r="F41" s="10"/>

</xml_diff>